<commit_message>
Ser ut til å virke med fartsgrenseanalyse
</commit_message>
<xml_diff>
--- a/Data/Hamar/om_sl_segments.xlsx
+++ b/Data/Hamar/om_sl_segments.xlsx
@@ -17850,7 +17850,7 @@
         <v>704826</v>
       </c>
       <c r="F458">
-        <v>0.1984232</v>
+        <v>0.20132718</v>
       </c>
       <c r="G458">
         <v>0.25578707</v>
@@ -35178,7 +35178,7 @@
         <v>0</v>
       </c>
       <c r="G1007">
-        <v>0.18371129</v>
+        <v>0.12264333</v>
       </c>
       <c r="I1007" t="s">
         <v>951</v>
@@ -50759,7 +50759,7 @@
         <v>0</v>
       </c>
       <c r="G1497">
-        <v>0.2733953</v>
+        <v>0.20897689</v>
       </c>
       <c r="I1497" t="s">
         <v>951</v>
@@ -53383,7 +53383,7 @@
         <v>0.22677348</v>
       </c>
       <c r="G1579">
-        <v>0.39369591</v>
+        <v>0.31258112</v>
       </c>
       <c r="I1579" t="s">
         <v>952</v>
@@ -74937,10 +74937,10 @@
         <v>2823435</v>
       </c>
       <c r="F2258">
-        <v>0</v>
+        <v>0.59906517</v>
       </c>
       <c r="G2258">
-        <v>0.59906517</v>
+        <v>0.93125691</v>
       </c>
       <c r="I2258" t="s">
         <v>951</v>
@@ -93799,7 +93799,7 @@
         <v>0.71386134</v>
       </c>
       <c r="G2851">
-        <v>0.89343065</v>
+        <v>0.81829945</v>
       </c>
       <c r="I2851" t="s">
         <v>951</v>

</xml_diff>